<commit_message>
chore: remove ai_workspace sandbox module and test junk
Deleted:
- ai_workspace/ — full Flask sandbox app (routes, tools, memory, web UI)
- ai_chat.py, ai_insights.json, ai_sessions.json — orphaned sandbox artifacts
- run_sandbox.bat — sandbox runner
- ai_workspace* broken dirs (analysisexports, analysisreports, logs, routes)

Core files (server.js dashboard.html labo_gui.py ai_*.py) are untouched
and remain functional on port 3000.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_thang/Thang_04_2026.xlsx
+++ b/Data_thang/Thang_04_2026.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J382"/>
+  <dimension ref="A1:J415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17854,6 +17854,1521 @@
         <v>3</v>
       </c>
       <c r="I382" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>263003039-1</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:54:00</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:00:00</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Tống Minh Luân</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:43-48, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H383" t="n">
+        <v>6</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Đắp hoàn tất</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Đã đóng gói chờ giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>262303048-4</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:50:00</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:00:00</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Trần V Ngãi</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:18-25, - SL: 13)</t>
+        </is>
+      </c>
+      <c r="H384" t="n">
+        <v>13</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Sửa Trực Trân</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Đã đóng gói chờ giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>262503048-2</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:47:00</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:00:00</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Nguyễn T Loan</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:15,23-27, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H385" t="n">
+        <v>6</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Sửa Trường Lân</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Đã đóng gói chờ giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>262703039-2</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:47:00</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:00:00</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Trần Văn Thanh</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:37-45, - SL: 12)</t>
+        </is>
+      </c>
+      <c r="H386" t="n">
+        <v>12</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>LTTS
+Đạt</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Đã đóng gói chờ giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>263003040-1</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:41:00</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:00:00</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Kim Quỳnh</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:22-23, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H387" t="n">
+        <v>2</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Hoàn tất. GẤP</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Đã đóng gói chờ giao</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>262903047-2</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:17:00</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:00:00</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:00:00</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>SG-Nk  Anh Khôi</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Chúc (Trúc)</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:15-22,33-36, - SL: 11)</t>
+        </is>
+      </c>
+      <c r="H388" t="n">
+        <v>11</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Sửa : Trang Trân
+BOOK GRAB NK TRẢ TIỀN</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>262803021-1</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2026-04-01 13:47:00</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:00:00</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:00:00</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Cô Hoa (38471)</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>Răng sứ Chrome - Cobalt (R:35-37,44, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H389" t="n">
+        <v>4</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Sửa Vy Hữu</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>262903029-1</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:21:00</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:00:00</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Anh Trung (47242)</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:34, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H390" t="n">
+        <v>1</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Sửa Trang Hữu</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>00703036-1</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2026-04-01 13:17:00</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Lê Thị Xuyên</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:32-42, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H391" t="n">
+        <v>4</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>BHHT CS1
+Vạn Tâm Trọng Nhuần Linh
+Giấy: 10h30 ngày 3/4 c gom</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>260104046</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2026-04-01 13:08:00</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Huỳnh Thị Kim Loan</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:14-23, - SL: 7)</t>
+        </is>
+      </c>
+      <c r="H392" t="n">
+        <v>7</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Hoàn tất - CS1
+Giấy 10h30 ngày 3/4 c gom</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>260104045</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2026-04-01 13:05:00</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Lê Thanh Tú</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Răng sứ Zir- Diamond (R:25-26, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H393" t="n">
+        <v>2</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>HT - CS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>260104051</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2026-04-01 15:06:00</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>SG-Nk  Hậu - Bình Chánh</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Chiến</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Răng sứ Zolid (R:12-22, - SL: 4); 
+Răng Tạm (R:12-22, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H394" t="n">
+        <v>8</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>TS 
+Đã tách giấy</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>262703048-2</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2026-04-01 14:50:00</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>LA-Nk Tố Oanh</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Nguyễn Hải Yến</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Full Sứ Ziconia (R:16, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H395" t="n">
+        <v>1</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>LLHT Trang Trân</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>262903038-1</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2026-04-01 11:33:00</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>2026-04-02 15:00:00</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:00:00</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>AG-Nk Hồng Thọ</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Ngọc Như</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11,21, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H396" t="n">
+        <v>2</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Sửa Trang Trân
+ĐÃ HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>260104023</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:10:00</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>AG-Nk Hiệp Thành</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Cùi giả (R:11,13, - SL: 2); 
+Răng sứ kim loại thường (R:11-13, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H397" t="n">
+        <v>5</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>260104028</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:18:00</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Tuyền</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:23,43,44-45,47, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H398" t="n">
+        <v>5</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>260104026</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:15:00</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Hoàng Anh</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:11,12,21,22, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H399" t="n">
+        <v>4</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>260104033</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:34:00</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>AG-Nk An Châu</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Ngô Thị Kim Tuyết</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:14-15, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H400" t="n">
+        <v>2</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>260104032</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:35:00</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>AG-Nk Nguyễn Gia</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Trần Thị Kim Ngọc</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11, - SL: 1); 
+Răng sứ Titanium (R:48, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H401" t="n">
+        <v>2</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>260104031</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:33:00</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>AG-Nk Nguyễn Gia</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Hồ Phú Lực</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12-21, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H402" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>263003030-1</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:31:00</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>AG-Nk An Châu</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Hà Thanh Tâm</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:14-15, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H403" t="n">
+        <v>2</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>32109010-1</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>2026-04-01 09:45:00</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>AG-Nk Thanh Bình</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Út Nal</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:34, - SL: 1); 
+Răng sứ kim loại thường (R:11, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H404" t="n">
+        <v>2</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>LHHT 11: Trí Gấm Trọng Vy Phú
+R34 sửa</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>261903053-1</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>2026-04-01 10:27:00</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:00:00</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Chị Phượng (37095)</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:44-47, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H405" t="n">
+        <v>4</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Sửa My Trân</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>262503063-2</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>2026-04-01 17:22:00</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:00:00</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Anh Tuấn (43918)</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:27-28,34-36, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H406" t="n">
+        <v>5</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>LLHT Trang Hỷ</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>260104044</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>2026-04-01 12:40:00</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>2026-04-03 08:00:00</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Chị Mai (47294)</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:35-37, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H407" t="n">
+        <v>3</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>ht</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>260104052</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026-04-01 16:00:00</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>2026-04-03 08:00:00</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>SG-Nk  An Dương Vương</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Phan Thị Kim Cương</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:24, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H408" t="n">
+        <v>1</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>241106026-3</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>2026-04-01 12:47:00</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>2026-04-03 09:00:00</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>SG-Nk Như Lạc</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Bác Ngọ</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:16, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H409" t="n">
+        <v>1</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Sửa Hồng Trân</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>260104053</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>2026-04-01 17:26:00</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>2026-04-03 10:00:00</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>2026-04-03 11:00:00</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>SG-Nk Mỹ Á</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Cô Tú</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:22, - SL: 1); 
+Răng Tạm (R:32-42, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H410" t="n">
+        <v>5</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>HT
+Đã tách giấy</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>260104047</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>2026-04-01 13:24:00</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>2026-04-03 10:00:00</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>LA-Nk Kim Oanh</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Tuyền</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:43-45, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H411" t="n">
+        <v>3</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>HT
+ĐÃ HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>260104055</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:55:00</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>2026-04-03 13:00:00</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Cô Anh (46784)</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:44, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H412" t="n">
+        <v>1</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>260104050</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>2026-04-01 14:05:00</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Cao Thanh Thuỷ</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:16-24,25-26,17, - SL: 13)</t>
+        </is>
+      </c>
+      <c r="H413" t="n">
+        <v>13</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>HT CS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>260104049</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>2026-04-01 14:00:00</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Trịnh Thị Ngọc Thuý</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:34-38,33, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H414" t="n">
+        <v>6</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>HT - CS 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>260104054</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>2026-04-01 18:50:00</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Anh Thái (47219)</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:21-22,23,24-27,15,32-42,33-34,35-38, - SL: 19)</t>
+        </is>
+      </c>
+      <c r="H415" t="n">
+        <v>19</v>
+      </c>
+      <c r="I415" t="inlineStr">
         <is>
           <t>HT</t>
         </is>

</xml_diff>

<commit_message>
chore: update last run file and add local shell permissions
- Point labo_config to Thang_04_2026 data file
- Add localhost/server startup shell permissions to local settings

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_thang/Thang_04_2026.xlsx
+++ b/Data_thang/Thang_04_2026.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J415"/>
+  <dimension ref="A1:J476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -19369,6 +19369,2765 @@
         <v>19</v>
       </c>
       <c r="I415" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>263103055-1</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:56:00</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>2026-04-02 12:00:00</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:00:00</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>SG-Nk  Hậu - Bình Chánh</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Loan</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Máng tẩy mềm 1.0mm (R:HTren,HDuoi, - SL: 1); 
+Răng sứ kim loại thường (R:45-46, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H416" t="n">
+        <v>3</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Đắp HT 
+Đã tách giấy</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>260104057</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>2026-04-01 19:08:00</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>2026-04-03 08:00:00</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>SG-Nk Huỳnh Lê</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Hồng Thu (14744)</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:32-33,31-42, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H417" t="n">
+        <v>5</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>262703029-1</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:37:00</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>AG-Nk Nguyễn Gia</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Trần Thị Thuý Hằng</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11-12, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H418" t="n">
+        <v>2</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Sửa Trang - Lân</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>263003019-1</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:34:00</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>NT-Nk BS Thuận</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Phạm Hải</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Full/ mão kim loại sứ titan (R:48, - SL: 1); 
+Răng sứ Titanium (R:45-47, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H419" t="n">
+        <v>4</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Sửa Hồng - Hỷ</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>262603026-1</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:29:00</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>NT-Nk BS Thuận</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Phong</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:11-12, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H420" t="n">
+        <v>2</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Sửa Hồng - Tuấn</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>261803018-1</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:50:00</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>BL-NK BS Tăng Suy Nghĩ</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Nguyễn Linh Phương</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:31-44, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H421" t="n">
+        <v>6</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Sửa (Trang-Hỷ)
+KHÔNG HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>260204003</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:43:00</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:00:00</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>BL-NK BS Tăng Suy Nghĩ</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Phan Thị Bé Lai</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:34-36, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H422" t="n">
+        <v>3</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>HT - GẤP. KHÔNG HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>262803030-2</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:22:00</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:00:00</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Nguyễn T Hường</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:23-24, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H423" t="n">
+        <v>2</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Sửa (Trang-Tuấn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>263103036-1</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:50:00</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:00:00</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Cao T Ren</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:22, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H424" t="n">
+        <v>1</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>HT
+GẤP - KHÔNG HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>263103035-1</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:45:00</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:00:00</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Phan Thị Bé Sáu</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:24-27, - SL: 4); 
+Răng sứ Titanium (R:35-36, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H425" t="n">
+        <v>6</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Đắp HT + LTHT 
+GẤP. KHÔNG HẸN</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>260204041</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:34:00</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>2026-04-03 08:00:00</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>TN-Nk  NHO</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>A. Liêm</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:34, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H426" t="n">
+        <v>1</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>263103045-1</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:10:00</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>2026-04-03 09:00:00</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>SG-Nk  An Dương Vương</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Võ Thị Phượng</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:33-37, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H427" t="n">
+        <v>5</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Đắp HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>262603037-2</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:43:00</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>2026-04-03 10:00:00</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>LA-Nk Tâm Đức</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Gái</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại  trên khung (R:35-37,45-47, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H428" t="n">
+        <v>6</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>LT - đắp hoàn tất
+Vy - Tuấn</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>262603038-2</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:49:00</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>2026-04-03 10:00:00</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>LA-Nk Tâm Đức</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Chính</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:16-26, - SL: 12)</t>
+        </is>
+      </c>
+      <c r="H429" t="n">
+        <v>12</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Sửa KHÔNG HẸN
+Vy - Trân</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>260204059</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:07:00</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>SG-Nk  Hậu - Bình Chánh</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Ngọc Bich</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:26, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H430" t="n">
+        <v>1</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>260204007</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:00:00</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>CT-NK Thanh Tú</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Phan T Bích Ngân</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:11,21, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H431" t="n">
+        <v>2</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>260204009</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:03:00</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>AG-Nk Thủy Tùng</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Sithon</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:46, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H432" t="n">
+        <v>1</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>260204008</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:58:00</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>AG-Nk Thủy Tùng</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Tân Thanh</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>Răng sứ Cercon HT (R:37, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H433" t="n">
+        <v>1</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>260204040</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:32:00</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>AG-Nk Hồng Thọ</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Nguyễn T Thu</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:16,36, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H434" t="n">
+        <v>2</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>260204013</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:09:00</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>TV-Nk Đức Hiền</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Chị Trang</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:43-47, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H435" t="n">
+        <v>5</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>260204011</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:05:00</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>DT-Nk BS Lê Văn Đệ</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Phạm Thị Thu Trang</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11-21, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H436" t="n">
+        <v>2</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>260204017</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:20:00</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>AG-Nk Hoàng Phương</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Diệu</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12-21, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H437" t="n">
+        <v>3</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>260204016</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:18:00</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>AG-Nk Thanh Quang</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Hằng</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:22-23, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H438" t="n">
+        <v>2</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>260204015</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:17:00</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>TV-Nk Đức Hiền</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Cô Trang</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H439" t="n">
+        <v>1</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>260204019</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:24:00</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>AG-Nk Hoàng Phương</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:22, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H440" t="n">
+        <v>1</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>260204032</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:59:00</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>BL-Nk Bs Quân</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Sơn Thị Bích Thuỷ</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Răng sứ Zir- Diamond (R:43-46, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H441" t="n">
+        <v>4</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>262903006-1</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:26:00</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>AG-Nk Thủy Tùng</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Cẩm Thy</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Răng sứ Cercon HT (R:45, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H442" t="n">
+        <v>1</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Sửa Vy - ko tên</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>260204026</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:45:00</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>AG-Nk Mai Thư- AP</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Lan</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:15-25, - SL: 10)</t>
+        </is>
+      </c>
+      <c r="H443" t="n">
+        <v>10</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>HT
+GỬI SỔ ĐẶT HÀNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>260204025</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:42:00</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>TV-Nk Thuấn Thư</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Trần Ngọc Thuý</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:33,44, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H444" t="n">
+        <v>2</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>260204021</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:28:00</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>AG-Nk Thanh Bình</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Phú Quốc</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:34-35, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H445" t="n">
+        <v>2</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>260204022</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:31:00</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>AG-Nk Thanh Bình</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Tuyết</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:43-47, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H446" t="n">
+        <v>5</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>260204030</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:54:00</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>NT-Nk BS Thuận</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Nguyễn Quá</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Răng sứ Cercon HT (R:13, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H447" t="n">
+        <v>1</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>260204029</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:51:00</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>AG-Nk Nguyễn Gia</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Lê Thị Ngọc Quyên</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:46-47, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H448" t="n">
+        <v>2</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>260204028</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:49:00</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>AG-Nk An Châu</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Trần Nhựt Em</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:34-35, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H449" t="n">
+        <v>2</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>251209054-3</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:04:00</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>AG-Nk Hiệp Hùng</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Phạm Thị Tâm</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12-22, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H450" t="n">
+        <v>4</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>BHHT (Phong-Sáng-Sĩ-Vy-Trân)</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>260204014</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:11:00</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>DL-Nk Đức Trọng</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Huy</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:26, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H451" t="n">
+        <v>1</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>260204010</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:15:00</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>DL-Nk Đức Trọng</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Uyên</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>Mặt dán sứ (R:12,22, - SL: 2); 
+Veneer sứ Ziconia (Cut Back) (R:11,21, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H452" t="n">
+        <v>4</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>260204012</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>2026-04-02 08:08:00</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>DL-Nk Đức Trọng</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Duy</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:37, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H453" t="n">
+        <v>1</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>260204006</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:53:00</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>KG-Nk Phạm Kiều</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Thuỷ</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại đắp sứ VITA (R:23-25, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H454" t="n">
+        <v>3</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>260204005</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:51:00</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>KG-Nk Phạm Kiều</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Mến</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại đắp sứ VITA (R:21, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H455" t="n">
+        <v>1</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>260204004</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:46:00</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>KG-Nk Phạm Kiều</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Phạm Thị Tưởng</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:43-44, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H456" t="n">
+        <v>2</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>260204039</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:30:00</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>AG-Nk Quốc Huy</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Út Hồng</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:34-35, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H457" t="n">
+        <v>2</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>262503024-1</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:10:00</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>AG-Nk Thanh Bình</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Bích Thuỷ</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>Full Sứ Ziconia (R:16-17,26, - SL: 3); 
+Răng sứ Zircornia (R:13-15,24-25, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H458" t="n">
+        <v>8</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>LLHT (Trường-Tuấn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>260204043</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:40:00</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Văn Phúc</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:14-16, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H459" t="n">
+        <v>3</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>260204045</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:43:00</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Cẩm Thuý</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:17,25,27, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H460" t="n">
+        <v>3</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>260204048</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:47:00</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>My Nhiên</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:25, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H461" t="n">
+        <v>1</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>260204047</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:45:00</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>ST-Nk BS Thùy</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Diệu Hiền</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:14, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H462" t="n">
+        <v>1</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>260204002</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:40:00</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>BL-NK BS Tăng Suy Nghĩ</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Đôi</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:35, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H463" t="n">
+        <v>1</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>260204001</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>2026-04-02 07:37:00</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:30:00</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>BL-NK BS Tăng Suy Nghĩ</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Trương Thị Tiếng</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12,25-27,35-38, - SL: 8)</t>
+        </is>
+      </c>
+      <c r="H464" t="n">
+        <v>8</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>262903043-2</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:13:00</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>2026-04-03 19:00:00</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Hồng Hiếu</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:14-15,25, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H465" t="n">
+        <v>3</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>LTHT (Vy-Tuấn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>260204060</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:09:00</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>2026-04-03 19:00:00</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Võ Thị Thanh Tuyến</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12,34-38,44-45, - SL: 8)</t>
+        </is>
+      </c>
+      <c r="H466" t="n">
+        <v>8</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>262603041-1</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:01:00</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>2026-04-04 10:00:00</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>LA-Nk Tâm Đức</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Ngọc Trâm</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:15, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H467" t="n">
+        <v>1</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>LTHT
+Trực - Hỷ</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>92005059-04</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:38:00</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Đỗ Thị Hoài Phước</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:12-22, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H468" t="n">
+        <v>4</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>BHHT (Kten-Tâm-Tâm-Hân-Diễm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>260204046</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:43:00</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Lê T Mỹ Duyên</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H469" t="n">
+        <v>1</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>260204055</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:57:00</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>2026-04-04 10:00:00</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>LA-Nk Tâm Đức</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Phát</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:27, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H470" t="n">
+        <v>1</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Hoàn tất</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>260204051</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>2026-04-02 10:04:00</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Châu T Hồng Thắm</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:24-26, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H471" t="n">
+        <v>3</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>260204050</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:55:00</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Lâm T Phụng</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:31-33, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H472" t="n">
+        <v>3</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>242112043-1</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:55:00</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Trần T Loan</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:27, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H473" t="n">
+        <v>1</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>BHHT
+My - Thư</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>260204049</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:52:00</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Trần T Kim Phượng</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:13-14, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H474" t="n">
+        <v>2</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>260204044</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>2026-04-02 09:40:00</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Thụy</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Nguyễn T  Xuân Mai</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:35-37, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H475" t="n">
+        <v>3</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>260204058</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>2026-04-02 11:03:00</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>2026-04-04 15:00:00</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>SG-Nk Như Lạc</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Dư Chiêu Bảo</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>Veneer sứ Ziconia (Cut Back) (R:25, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H476" t="n">
+        <v>1</v>
+      </c>
+      <c r="I476" t="inlineStr">
         <is>
           <t>HT</t>
         </is>

</xml_diff>

<commit_message>
feat(mobile): glassmorphism dashboard redesign with smart time grouping
- Add dark glassmorphism CSS with stage-color accent bars (CBM/SAP/SUON/DAP/MAI)
- Add 8 JS helper functions: getNextActiveStageColor, isOverdue, classifyTimeGroup, smartSort, computeTimeGroups, renderOrderCard, tickCountdowns
- Replace mRender() with 3-pass pipeline: filter → smart group → render
- Smart grouping: auto-detects AM/PM presence from data, only shows existing groups
- Smart sorting: overdue first → fewest remaining stages → 15H urgency flag
- Live countdown every 60s (Còn Xh Yp / Trễ Xh Yp)
- Move filter chips to fixed bottom bar with safe-area-inset-bottom
- Header and KPI strip glassmorphism upgrade

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data_thang/Thang_04_2026.xlsx
+++ b/Data_thang/Thang_04_2026.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J476"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -22130,6 +22130,1091 @@
       <c r="I476" t="inlineStr">
         <is>
           <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>260204072</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:00:00</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>LA-Nk Tố Oanh</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Nguyễn Lê Quốc Duy</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Full sứ Cercon HT (R:36, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H477" t="n">
+        <v>1</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>260204067</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:23:00</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>DT- Nk BS Nhựt NM</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Ánh Nguyệt</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:12, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H478" t="n">
+        <v>1</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>263003046-1</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:30:00</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Nguyễn Trần Xuân Nhuỵ</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Răng sứ Zir- Diamond (R:31-41,32-33,42-43, - SL: 6)</t>
+        </is>
+      </c>
+      <c r="H479" t="n">
+        <v>6</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Sửa (Hồng-Tuấn)
+GỬI CS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>260204064</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:30:00</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Cao Quốc Dương</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Răng sứ Cercon HT (R:33-36, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H480" t="n">
+        <v>4</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>HT - GỬI CS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>260204063</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:30:00</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Nguyễn T Hồng Cẩm</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:11-21, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H481" t="n">
+        <v>2</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>HT - GỬI CS2</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>262803052-2</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:12:00</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>2026-04-03 12:00:00</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>LA-Nk Tố Oanh</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Thái Thị Đẹt</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:13-15, - SL: 3); 
+Veneer sứ Titanium (Cut Back) (R:12, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H482" t="n">
+        <v>4</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Sửa Trang Tuấn</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>260204075</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:32:00</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>LA-Nk  BS Thu</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Phạm T Kiều Chinh</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:12-21, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H483" t="n">
+        <v>3</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>262803058-1</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Ái</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Mỹ Dung</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:46, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H484" t="n">
+        <v>1</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>262903031-2</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:38:00</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>2026-04-03 15:00:00</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Anh Chung (47041)</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:35-37, - SL: 3)</t>
+        </is>
+      </c>
+      <c r="H485" t="n">
+        <v>3</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Sửa Vy Hữu</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>260204080</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:35:00</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>LA-Nk Khánh Hà</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Hồ Thị Kim Liên</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>Full Sứ Ziconia (R:36, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H486" t="n">
+        <v>1</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>262703057-4</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:11:00</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Ái</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Cao Thị Hồng Phượng</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:43-47, - SL: 5)</t>
+        </is>
+      </c>
+      <c r="H487" t="n">
+        <v>5</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Sửa Trường Trân gửi sổ chỉ định</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>262703057-3</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:15:00</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Ái</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Cao Thị Hồng Phượng</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:24-25, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H488" t="n">
+        <v>2</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>LT Thử thô Trường Trân</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>260204076</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:36:00</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>2026-04-03 14:00:00</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Cẩm Dung</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Bé Nhi</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:26, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H489" t="n">
+        <v>1</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>260204069</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:25:00</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>2026-04-03 16:00:00</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Cô Cương (41654)</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:34, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H490" t="n">
+        <v>1</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>262803053-2</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>SG-Nk Việt Xuân</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Thu Huỳnh</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>Răng sứ Zircornia (R:17, - SL: 1); 
+Răng sứ Zircornia (R:46, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H491" t="n">
+        <v>2</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>R17: sửa
+R46: LTHT VY TRÂN</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>260104041-1</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:22:00</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>2026-04-03 17:00:00</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Chú Cửu (47284)</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:38, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H492" t="n">
+        <v>1</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>260204068</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>2026-04-02 14:41:00</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>2026-04-03 19:00:00</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>BT-Nk Bác Sĩ Hiếu</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Nguyễn Cao Thái Long</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:46, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H493" t="n">
+        <v>1</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>260204074</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:30:00</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>2026-04-04 08:00:00</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>SG-Nk Việt Xuân</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Lữ Thị Hồng Oanh</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:43, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H494" t="n">
+        <v>1</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>260204071</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:26:00</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>2026-04-03 18:00:00</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>2026-04-04 10:00:00</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>SG-Nk  Anh Khôi</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Phương</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:37, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H495" t="n">
+        <v>1</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>260204070</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:24:00</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>2026-04-04 13:00:00</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Hiền (47319)</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>Răng sứ Chrome - Cobalt (R:36, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H496" t="n">
+        <v>1</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>260204078</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-04-02 19:25:00</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>2026-04-04 13:00:00</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>SG-Nk Hải Nguyên</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Thầy Thanh (47296)</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>Răng sứ Titanium (R:36,45-47, - SL: 4)</t>
+        </is>
+      </c>
+      <c r="H497" t="n">
+        <v>4</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>HT</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>260204062</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:30:00</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Lê Văn Thanh</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>Răng sứ kim loại thường (R:35-36, - SL: 2)</t>
+        </is>
+      </c>
+      <c r="H498" t="n">
+        <v>2</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>HT - GỬI CS1</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>251011044-2</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2026-04-02 13:00:00</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>2026-04-04 12:00:00</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Huý</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Võ Chí Cường</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>Răng sứ Zir- Diamond (R:15-17,11,21,22,23-26, - SL: 10)</t>
+        </is>
+      </c>
+      <c r="H499" t="n">
+        <v>10</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>BHHT (Vạn-Nha Việt x2-Hồng-Tuấn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>262503058-1</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:30:00</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>2026-04-04 14:00:00</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>2026-04-04 16:00:00</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>LA-Nk BS Cẩm Dung</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Chị Thuý</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>Inlay/Onlay/Overlay  kim loại thường (R:17, - SL: 1); 
+Răng sứ Zircornia (R:24, - SL: 1)</t>
+        </is>
+      </c>
+      <c r="H500" t="n">
+        <v>2</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>HT ĐÃ HẸN</t>
         </is>
       </c>
     </row>

</xml_diff>